<commit_message>
Add Week 2 market intelligence and KSCP financial analysis
</commit_message>
<xml_diff>
--- a/W02_Market_Data.xlsx
+++ b/W02_Market_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\大王只想要工作\intern\Week 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A43C0B3C-F84D-421D-AD0F-37EC0378127B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCD6C1B-964A-46A7-B39B-E965274A8237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1605" yWindow="1845" windowWidth="23685" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12360" yWindow="1950" windowWidth="26205" windowHeight="18420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Company_Comparison" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="118">
   <si>
     <t>Company</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -186,12 +186,6 @@
   </si>
   <si>
     <t>Includes military and defense applications in addition to commercial security robotics, so the estimate is broader than InGen’s patrol and enterprise security use cases. Detailed underlying data are paywalled.</t>
-  </si>
-  <si>
-    <t>Service Robotics Market Size And Share Report, 2024-2030</t>
-  </si>
-  <si>
-    <t>Security Robots Market Size And Share Report, 2024-2030</t>
   </si>
   <si>
     <t>Autonomous physical security / security robotics</t>
@@ -230,10 +224,6 @@
     <t>10,000+ figure includes stationary devices, robots, and agents; it should not be interpreted as 10,000 deployed ASRs.</t>
   </si>
   <si>
-    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465926036240/kscp-20251231x10k.htm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Eldercare / AI companion robotics</t>
   </si>
   <si>
@@ -247,9 +237,6 @@
     <t>ElliQ</t>
   </si>
   <si>
-    <t>Thousands of older adults in the U.S.; exact unit count not disclose</t>
-  </si>
-  <si>
     <t>Proprietary Relationship Orchestrator integrating multiple LLMs, contextual memory, emotional-state estimation, multimodal interaction, and proactive decision-making</t>
   </si>
   <si>
@@ -364,82 +351,96 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>Q1 2026</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Knightscope Form 10-Q, quarter ended March 31, 2026</t>
+  </si>
+  <si>
+    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465926062505/kscp-20260331x10q.htm</t>
+  </si>
+  <si>
+    <t>Q1 2026 includes approximately $2.4M of Security Force revenue following the KSF acquisition completed on February 27, 2026.</t>
+  </si>
+  <si>
+    <t>Q4 2025</t>
+  </si>
+  <si>
+    <t>Knightscope FY2025 Form 10-K + Q3 2025 Form 10-Q</t>
+  </si>
+  <si>
+    <t>Q4 income-statement and operating cash burn figures are derived as FY2025 less the nine months ended Sep. 30, 2025. Cash balance is directly reported as of Dec. 31, 2025.</t>
+  </si>
+  <si>
+    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465926036240/kscp-20251231x10k.htm,https://www.sec.gov/Archives/edgar/data/1600983/000110465925110518/kscp-20250930x10q.htm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q3 2025</t>
+  </si>
+  <si>
+    <t>Q2 2025</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Q1 2025</t>
+  </si>
+  <si>
+    <t>Knightscope Q1 2025 Form 10-Q</t>
+  </si>
+  <si>
+    <t>https://www.sec.gov/Archives/edgar/data/1600983/000155837025007781/kscp-20250331x10q.htm</t>
+  </si>
+  <si>
+    <t>SG&amp;A combines reported Sales &amp; Marketing and General &amp; Administrative expenses.</t>
+  </si>
+  <si>
+    <t>Knightscope Q2 2025 Form 10-Q</t>
+  </si>
+  <si>
+    <t>https://www.sec.gov/Archives/edgar/data/1600983/000155837025011247/kscp-20250630x10q.htm</t>
+  </si>
+  <si>
+    <t>Quarterly cash burn derived as H1 2025 operating cash used less Q1 2025 operating cash used.</t>
+  </si>
+  <si>
+    <t>Knightscope Q3 2025 Form 10-Q</t>
+  </si>
+  <si>
+    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465925110518/kscp-20250930x10q.htm</t>
+  </si>
+  <si>
+    <t>Quarterly cash burn derived as 9M 2025 operating cash used less H1 2025 operating cash used.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.grandviewresearch.com/industry-analysis/service-robotics-industry</t>
+  </si>
+  <si>
+    <t>27-Mar-26 (10-K); 12-Nov-25 (Q3 10-Q)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Thousands of older adults in the U.S.; exact unit count not disclosed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465926094859/kscp-20260630x10q.htm</t>
-  </si>
-  <si>
-    <t>Q1 2026</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Knightscope Form 10-Q, quarter ended March 31, 2026</t>
-  </si>
-  <si>
-    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465926062505/kscp-20260331x10q.htm</t>
-  </si>
-  <si>
-    <t>Q1 2026 includes approximately $2.4M of Security Force revenue following the KSF acquisition completed on February 27, 2026.</t>
-  </si>
-  <si>
-    <t>Q4 2025</t>
-  </si>
-  <si>
-    <t>Knightscope FY2025 Form 10-K + Q3 2025 Form 10-Q</t>
-  </si>
-  <si>
-    <t>27-Mar-26 (10-K)</t>
-  </si>
-  <si>
-    <t>Q4 income-statement and operating cash burn figures are derived as FY2025 less the nine months ended Sep. 30, 2025. Cash balance is directly reported as of Dec. 31, 2025.</t>
-  </si>
-  <si>
-    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465926036240/kscp-20251231x10k.htm,https://www.sec.gov/Archives/edgar/data/1600983/000110465925110518/kscp-20250930x10q.htm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Q3 2025</t>
-  </si>
-  <si>
-    <t>Q2 2025</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Q1 2025</t>
-  </si>
-  <si>
-    <t>Knightscope Q1 2025 Form 10-Q</t>
-  </si>
-  <si>
-    <t>https://www.sec.gov/Archives/edgar/data/1600983/000155837025007781/kscp-20250331x10q.htm</t>
-  </si>
-  <si>
-    <t>SG&amp;A combines reported Sales &amp; Marketing and General &amp; Administrative expenses.</t>
-  </si>
-  <si>
-    <t>Knightscope Q2 2025 Form 10-Q</t>
-  </si>
-  <si>
-    <t>https://www.sec.gov/Archives/edgar/data/1600983/000155837025011247/kscp-20250630x10q.htm</t>
-  </si>
-  <si>
-    <t>Quarterly cash burn derived as H1 2025 operating cash used less Q1 2025 operating cash used.</t>
-  </si>
-  <si>
-    <t>Knightscope Q3 2025 Form 10-Q</t>
-  </si>
-  <si>
-    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465925110518/kscp-20250930x10q.htm</t>
-  </si>
-  <si>
-    <t>Quarterly cash burn derived as 9M 2025 operating cash used less H1 2025 operating cash used.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.sec.gov/Archives/edgar/data/1600983/000110465926036240/kscp-20251231x10k.htm; https://www.sec.gov/Archives/edgar/data/1600983/000110465926094859/kscp-20260630x10q.htm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="26" formatCode="\$#,##0.00_);[Red]\(\$#,##0.00\)"/>
-  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -493,12 +494,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="26" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -839,34 +839,34 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C2">
         <v>2013</v>
       </c>
       <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" t="s">
         <v>51</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>52</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>53</v>
       </c>
-      <c r="G2" t="s">
-        <v>54</v>
-      </c>
-      <c r="H2" t="s">
-        <v>55</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>57</v>
+        <v>117</v>
       </c>
       <c r="J2" s="1">
         <v>46280</v>
       </c>
       <c r="K2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -874,69 +874,69 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C3">
         <v>2016</v>
       </c>
       <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" t="s">
+        <v>115</v>
+      </c>
+      <c r="H3" t="s">
         <v>59</v>
       </c>
-      <c r="E3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="I3" t="s">
         <v>61</v>
-      </c>
-      <c r="G3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H3" t="s">
-        <v>63</v>
-      </c>
-      <c r="I3" t="s">
-        <v>65</v>
       </c>
       <c r="J3" s="1">
         <v>46280</v>
       </c>
       <c r="K3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C4">
         <v>1990</v>
       </c>
       <c r="D4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" t="s">
+        <v>67</v>
+      </c>
+      <c r="H4" t="s">
         <v>68</v>
       </c>
-      <c r="E4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="I4" t="s">
         <v>70</v>
-      </c>
-      <c r="G4" t="s">
-        <v>71</v>
-      </c>
-      <c r="H4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I4" t="s">
-        <v>74</v>
       </c>
       <c r="J4" s="1">
         <v>46280</v>
       </c>
       <c r="K4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -944,75 +944,75 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C5">
         <v>2016</v>
       </c>
       <c r="D5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>74</v>
+      </c>
+      <c r="G5" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" t="s">
         <v>76</v>
       </c>
-      <c r="E5" t="s">
-        <v>77</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="I5" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="G5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H5" t="s">
-        <v>80</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="J5" s="1">
         <v>46280</v>
       </c>
       <c r="K5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C6">
         <v>2012</v>
       </c>
       <c r="D6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" t="s">
         <v>85</v>
       </c>
-      <c r="E6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="I6" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="G6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H6" t="s">
-        <v>89</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="J6" s="1">
         <v>46280</v>
       </c>
       <c r="K6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{2A4347B1-598A-475A-980E-CBF15E1BBCAA}"/>
+    <hyperlink ref="I2" r:id="rId1" display="https://www.sec.gov/Archives/edgar/data/1600983/000110465926036240/kscp-20251231x10k.htm" xr:uid="{2A4347B1-598A-475A-980E-CBF15E1BBCAA}"/>
     <hyperlink ref="I5" r:id="rId2" xr:uid="{79640ABA-8C36-411E-B36D-38EF96F9AE8E}"/>
     <hyperlink ref="I6" r:id="rId3" xr:uid="{2A1EB646-8369-4832-89B0-D33B6A2A62EA}"/>
   </hyperlinks>
@@ -1026,6 +1026,11 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="11.625" customWidth="1"/>
+    <col min="4" max="4" width="12.125" customWidth="1"/>
+    <col min="5" max="5" width="10.875" customWidth="1"/>
+    <col min="6" max="6" width="10.625" customWidth="1"/>
     <col min="7" max="7" width="11.25" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1034,22 +1039,22 @@
         <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C1" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="F1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1111,7 +1116,7 @@
       <c r="D4">
         <v>-1.57</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4">
         <v>-1.619</v>
       </c>
       <c r="F4">
@@ -1169,7 +1174,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B7">
         <v>4.0350000000000001</v>
@@ -1207,7 +1212,7 @@
         <v>20.565999999999999</v>
       </c>
       <c r="F8">
-        <v>11.4</v>
+        <v>11.401</v>
       </c>
       <c r="G8">
         <v>8.16</v>
@@ -1230,30 +1235,33 @@
         <v>10.61</v>
       </c>
       <c r="F9">
-        <v>11.6</v>
+        <v>11.603999999999999</v>
+      </c>
+      <c r="G9" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>60</v>
+      <c r="B10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1261,22 +1269,22 @@
         <v>25</v>
       </c>
       <c r="B11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" t="s">
         <v>109</v>
       </c>
-      <c r="C11" t="s">
-        <v>112</v>
-      </c>
-      <c r="D11" t="s">
-        <v>115</v>
-      </c>
       <c r="E11" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F11" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="G11" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1293,7 +1301,7 @@
         <v>45973</v>
       </c>
       <c r="E12" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="F12" s="1">
         <v>46157</v>
@@ -1307,22 +1315,22 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" t="s">
         <v>110</v>
       </c>
-      <c r="C13" t="s">
-        <v>113</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="E13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F13" t="s">
+        <v>94</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F13" t="s">
-        <v>99</v>
-      </c>
-      <c r="G13" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1330,28 +1338,29 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" t="s">
+        <v>108</v>
+      </c>
+      <c r="D14" t="s">
         <v>111</v>
       </c>
-      <c r="C14" t="s">
-        <v>114</v>
-      </c>
-      <c r="D14" t="s">
-        <v>117</v>
-      </c>
       <c r="E14" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F14" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G14" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="E13" r:id="rId1" xr:uid="{5D3059AC-C792-42F1-AE26-DCFD24D55FEA}"/>
+    <hyperlink ref="G13" r:id="rId2" xr:uid="{4212C370-FB5F-41A6-A988-F49DE32781E3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1369,7 +1378,7 @@
     <col min="5" max="5" width="65.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="54.25" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1425,7 +1434,7 @@
         <v>46</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>48</v>
+        <v>113</v>
       </c>
       <c r="I2" s="1">
         <v>46280</v>
@@ -1435,6 +1444,9 @@
       <c r="A3" t="s">
         <v>39</v>
       </c>
+      <c r="B3" t="s">
+        <v>112</v>
+      </c>
       <c r="C3" t="s">
         <v>36</v>
       </c>
@@ -1446,6 +1458,12 @@
       </c>
       <c r="F3" t="s">
         <v>41</v>
+      </c>
+      <c r="G3" t="s">
+        <v>112</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>113</v>
       </c>
       <c r="I3" s="1">
         <v>46280</v>
@@ -1474,7 +1492,7 @@
         <v>47</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="I4" s="1">
         <v>46280</v>
@@ -1483,8 +1501,9 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" display="https://www.grandviewresearch.com/industry-analysis/service-robotics-industry" xr:uid="{3893008C-C864-412D-AA73-551BA432C82E}"/>
-    <hyperlink ref="H4" r:id="rId2" display="https://www.grandviewresearch.com/industry-analysis/security-robots-market-report" xr:uid="{C0DCABAA-A743-41C9-B8CA-4A789E8BBE40}"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{3893008C-C864-412D-AA73-551BA432C82E}"/>
+    <hyperlink ref="H3" r:id="rId2" xr:uid="{20D9ABF9-D3B6-4AAE-A825-A837964D3C3D}"/>
+    <hyperlink ref="H4" r:id="rId3" xr:uid="{8D28D9D2-5A1C-40C4-A057-D9B8A48DC9A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>